<commit_message>
Confirm male label for manuscript Table 1
</commit_message>
<xml_diff>
--- a/docs/manuscript_development/generated_assets/supplementary_etable1_2_cohort_characteristics.xlsx
+++ b/docs/manuscript_development/generated_assets/supplementary_etable1_2_cohort_characteristics.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,42 +431,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>table</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>characteristic</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Left SctO2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Right SctO2</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>SftO2</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Missing Left SctO2</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Missing Right SctO2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Missing SftO2</t>
         </is>
@@ -1296,7 +1308,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SEX, n (%)</t>
+          <t>Male, n (%)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2455,27 +2467,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>table</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>cohort</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>characteristic</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>missing_n</t>
         </is>
@@ -2919,7 +2931,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SEX, n (%)</t>
+          <t>Male, n (%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -4244,7 +4256,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SEX, n (%)</t>
+          <t>Male, n (%)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -5569,7 +5581,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>SEX, n (%)</t>
+          <t>Male, n (%)</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -6471,22 +6483,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ycol</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>n_rows</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>n_patients</t>
         </is>

</xml_diff>